<commit_message>
fix: distinguish Excel opening stock from purchases
</commit_message>
<xml_diff>
--- a/frontend/public/material-excel-en.xlsx
+++ b/frontend/public/material-excel-en.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb549ba411c584688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R56ae83d6fefb4318"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
   </x:cols>
@@ -344,10 +344,8 @@
           <x:t xml:space="preserve">Unit</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current Stock</x:t>
-        </x:is>
+      <x:c r="E1" t="str">
+        <x:v>Initial Stock (Not Purchase Receipt)</x:v>
       </x:c>
       <x:c r="F1" t="inlineStr">
         <x:is>

</xml_diff>